<commit_message>
Stage 2 results workbook: simplified wording, totals as values
Replace results/GLASS_Stage2_results.xlsx with the lead author's revised
version:
- three sheets (results per configuration, all 70 runs, settings and
  scoring); the findings stay in the results README;
- simplified column wording ("first proposal" / "after refinement");
- totals as plain numbers instead of formulas: valid 61 -> 66, all KPIs
  improved 35 -> 40, both 33 -> 38, refinement made it worse 22, and the
  per-KPI-type counts, all unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evaluation/loanapp_p2p/results/GLASS_Stage2_results.xlsx
+++ b/evaluation/loanapp_p2p/results/GLASS_Stage2_results.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results per configuration" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All 70 runs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings and scoring" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +40,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -82,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -94,6 +97,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -490,47 +499,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Valid (initial → final)</t>
+          <t>Valid scenario (first proposal → after refinement)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>All KPIs improved (initial → final)</t>
+          <t>All target KPIs improved (first proposal → after refinement)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Valid and improved (final)</t>
+          <t>Valid and all KPIs improved (after refinement)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Problems addressed (final)</t>
+          <t>Injected problems addressed (after refinement)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Precision (final)</t>
+          <t>Share of changes that target an injected problem (after refinement)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Recall (initial → final)</t>
+          <t>Share of injected changes recovered (first proposal → after refinement)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>CTD ratio (initial → final)</t>
+          <t>Closeness to the healthy model, 0 = no change, 1 = healthy (first proposal → after refinement)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Loop discarded a better initial</t>
+          <t>Runs where the refinement made the result worse than the first proposal</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Mean iterations</t>
+          <t>Refinement iterations used (mean)</t>
         </is>
       </c>
     </row>
@@ -1303,12 +1312,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Initial</t>
+          <t>First proposal</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>After refinement</t>
         </is>
       </c>
       <c r="D19" s="3" t="n"/>
@@ -1326,13 +1335,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="B20" s="2">
-        <f>COUNTIF('All 70 runs'!$G$2:$G$71,"yes")</f>
-        <v/>
-      </c>
-      <c r="C20" s="2">
-        <f>COUNTIF('All 70 runs'!$H$2:$H$71,"yes")</f>
-        <v/>
+      <c r="B20" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>66</v>
       </c>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -1349,13 +1356,11 @@
           <t>All KPIs improved</t>
         </is>
       </c>
-      <c r="B21" s="2">
-        <f>COUNTIF('All 70 runs'!$M$2:$M$71,"yes")</f>
-        <v/>
-      </c>
-      <c r="C21" s="2">
-        <f>COUNTIF('All 70 runs'!$N$2:$N$71,"yes")</f>
-        <v/>
+      <c r="B21" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>40</v>
       </c>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -1372,13 +1377,11 @@
           <t>Valid and all KPIs improved</t>
         </is>
       </c>
-      <c r="B22" s="2">
-        <f>COUNTIFS('All 70 runs'!$G$2:$G$71,"yes",'All 70 runs'!$M$2:$M$71,"yes")</f>
-        <v/>
-      </c>
-      <c r="C22" s="2">
-        <f>COUNTIFS('All 70 runs'!$H$2:$H$71,"yes",'All 70 runs'!$N$2:$N$71,"yes")</f>
-        <v/>
+      <c r="B22" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>38</v>
       </c>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -1400,9 +1403,8 @@
           <t>–</t>
         </is>
       </c>
-      <c r="C23" s="2">
-        <f>COUNTIF('All 70 runs'!$U$2:$U$71,"yes")</f>
-        <v/>
+      <c r="C23" s="2" t="n">
+        <v>22</v>
       </c>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -1416,7 +1418,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Formulas count the rows of sheet "All 70 runs" (Excel recalculates them on opening).</t>
+          <t>Totals are counts over the 70 runs (from the sheet 'All 70 runs').</t>
         </is>
       </c>
       <c r="B24" s="3" t="n"/>
@@ -1468,12 +1470,12 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Improved (initial)</t>
+          <t>Improved (first proposal)</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>Improved (final)</t>
+          <t>Improved (after refinement)</t>
         </is>
       </c>
       <c r="D27" s="3" t="n"/>
@@ -1576,6 +1578,36 @@
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
+      <c r="K32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>How to read: 'first proposal' = the scenario GLASS proposes first; 'after refinement' = the scenario GLASS selects after its simulation-based refinement (up to 4 iterations). Counts are out of 5 runs per configuration.</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+      <c r="K33" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1638,7 +1670,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Iterations used</t>
+          <t>Refinement iterations used</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1648,82 +1680,82 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Valid (initial)</t>
+          <t>Valid (first proposal)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Valid (final)</t>
+          <t>Valid (after refinement)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Violations (initial)</t>
+          <t>Violations (first proposal)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Violations (final)</t>
+          <t>Violations (after refinement)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>KPI change % (initial)</t>
+          <t>KPI change % (first proposal)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>KPI change % (final)</t>
+          <t>KPI change % (after refinement)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>All KPIs improved (initial)</t>
+          <t>All KPIs improved (first proposal)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>All KPIs improved (final)</t>
+          <t>All KPIs improved (after refinement)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Problems addressed (initial)</t>
+          <t>Problems addressed (first proposal)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Problems addressed (final)</t>
+          <t>Problems addressed (after refinement)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Recall (initial)</t>
+          <t>Injected changes recovered (first proposal)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Recall (final)</t>
+          <t>Injected changes recovered (after refinement)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>CTD ratio (initial)</t>
+          <t>Closeness to healthy (first proposal)</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>CTD ratio (final)</t>
+          <t>Closeness to healthy (after refinement)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Discarded better initial</t>
+          <t>Refinement made it worse</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Final modifications</t>
+          <t>Changes in the scenario after refinement</t>
         </is>
       </c>
     </row>
@@ -9175,130 +9207,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Finding</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>GLASS produces valid, KPI-improving scenarios for simple problems, but recovers only part of the injected causes.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Validity is high, and single-problem LoanApp configurations improve their KPI in nearly every run. Recall is mostly 0.06–0.25; the exception is LoanApp G3 (staffing), with recall 1.0 and CTD ratio 0.87. Typical pattern: one obvious activity shortened or one timer halved, plus extra staff, often in roles that were not affected, instead of reversing all injected changes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>GLASS's utilization metric makes the refinement loop discard correct fixes in congested configurations.</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>GLASS computes utilization as busy time ÷ the whole simulated span, so it rises when a fix clears a backlog. Under minimize, the feedback calls the correct fix a degradation. In LoanApp G1+G3 and G1+G2+G3, the initial patch (adding Loan Officers) reaches CTD ratio 0.96 / 0.88; the loop then picks near-no-op finals (CTD ratio about 0.0) in all 10 runs. Overall the loop discarded a better initial in 22 runs; in 15 of them GLASS's utilization rose while the pool's real utilization fell.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>The refinement loop helps in some configurations.</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>All KPIs improved, initial → final: LoanApp G2 3 → 4; Procure2Pay G1 1 → 3, G3 0 → 2, G1+G2 1 → 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Procure2Pay is harder than LoanApp.</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>In 5 runs iteration 1 failed GLASS's validator because the LLM used the resource-id stem QBP_DEFAULT_RESOURCE as a role name; later iterations succeeded and those finals were evaluated in the completion step. Two Procure2Pay G2 finals break the 35 % budget (+39 %): GLASS shows the limit to the LLM but only enforces absolute monthly budgets. No Procure2Pay configuration combining G1 and G3 is fully improved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Clarification context: the summariser fix holds in most cases.</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>GLASS re-summarises the chat, including the injected feedback, in every iteration, so the constraints block differs from iteration 1 in 86 of 98 later iterations, mostly in wording. In 4 of 168 summaries it still read "+3 per role" as a global cap of 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>The utilization limit is a sensitive choice.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>At 0.90 instead of 0.85, 22 instead of 18 initial scenarios count as improved; finals stay at 16.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>